<commit_message>
updated to new estimation strategy
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\simpaths_dev\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496F0204-32B2-4494-AB59-B58547A7709A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F518E279-5FED-44B4-840A-F9BBB1EBFF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -562,7 +562,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>7.4908409588260065</v>
+        <v>6.5883330217266201</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>